<commit_message>
Improve Lab 3 Excel starter and solution workbooks with full sheet templates.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data_platforms/production-support-day2/Lab_03_SLA_Reporting_Blameless_Postmortem/instructor/lab3_solution.xlsx
+++ b/data_platforms/production-support-day2/Lab_03_SLA_Reporting_Blameless_Postmortem/instructor/lab3_solution.xlsx
@@ -35,12 +35,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,8 +60,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,8 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -432,14 +444,19 @@
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ServiceHealth (1=up, 0=down)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ResponseTimeMs</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -455,6 +472,11 @@
       <c r="C2" t="n">
         <v>95</v>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Service up</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -468,6 +490,11 @@
       <c r="C3" t="n">
         <v>102</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Service up</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -483,6 +510,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Service down</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -498,6 +530,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Service down</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -511,6 +548,11 @@
       <c r="C6" t="n">
         <v>180</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Service up; slow response</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -523,6 +565,11 @@
       </c>
       <c r="C7" t="n">
         <v>88</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Service up</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -536,8 +583,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -545,17 +598,17 @@
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ServiceHealth</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ResponseTimeMs</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Exceeds 150ms SLA?</t>
         </is>
@@ -676,21 +729,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Total downtime (minutes)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>10</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Downtime intervals (5 min each)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Total downtime (minutes)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Response SLA compliance %</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>75</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Resolution SLA compliance %</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -704,77 +793,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Total time (minutes)</t>
-        </is>
-      </c>
-      <c r="B1" t="n">
-        <v>60</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Downtime (minutes)</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>10</v>
+          <t>Total time (minutes)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Observation window</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Uptime (minutes)</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>50</v>
+          <t>Downtime (minutes)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>From SLA Calculations</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Number of incidents</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>1</v>
+          <t>Uptime (minutes)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Total time − downtime</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MTTR (minutes)</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>10</v>
+          <t>Number of incidents</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Count downtime events</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MTBF (minutes)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50</v>
+          <t>MTTR (minutes)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Downtime ÷ incidents</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>MTBF (minutes)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Uptime ÷ failures</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Availability %</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>83.33</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>(Total − downtime) ÷ total × 100</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>83.33%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -788,8 +936,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -797,7 +949,7 @@
           <t>Metric</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -809,17 +961,39 @@
           <t>Availability %</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>83.33</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>83.33%</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>SLA target (99.9% max downtime/month, min)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>This incident downtime (min)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Meets 99.9% if only incident?</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -836,15 +1010,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>WEEKLY KPI DASHBOARD</t>
         </is>
       </c>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -852,35 +1031,213 @@
           <t>Date: 2026-06-10</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Service Availability: 83.33%</t>
-        </is>
-      </c>
+          <t>SERVICE HEALTH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Total Downtime (min): 10</t>
+          <t>Service Availability</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>83.33%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MTTR (min): 10</t>
-        </is>
+          <t>Total Downtime (min)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MTBF (min): 50</t>
+          <t>Number of Incidents</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SLA COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Response SLA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Resolution SLA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Overall SLA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>83.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RELIABILITY METRICS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MTTR (minutes)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MTBF (minutes)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TOP ALERTS</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Service Down</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>High Response Time</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ACTION ITEMS</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Add port-conflict check to deployment runbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Enable CloudWatch alarm → on-call for P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Schedule postmortem review within 48h</t>
         </is>
       </c>
     </row>
@@ -895,37 +1252,341 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>INC-AWS-001</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>BLAMELESS POSTMORTEM</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Incident ID: INC-AWS-001</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SERVICE</t>
+          <t>DATE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>payment-processor</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>SERVICE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>payment-processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SEVERITY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SLA MET?</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>No — 10 min downtime in sample window</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WHAT HAPPENED?</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rogue process held port 8080; payment-processor failed to start. CloudWatch ServiceHealth dropped to 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WHEN?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Start time</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>End time</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Duration (minutes)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>5 WHYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1. Why did the service fail?</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Port 8080 already in use</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2. Why did that happen?</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>rogue-process.py from Lab 2 setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3. Why did that happen?</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Not cleaned up after prior failure</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>4. Why did that happen?</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>No automated port check on service start</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5. Why did that happen?</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Runbook did not include ss/tulpn verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Root cause</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Port 8080 blocked by rogue-process.py</t>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Port conflict from orphaned rogue process; missing pre-start port validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WHAT WENT WELL?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CloudWatch alarm detected downtime quickly</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>WHAT WENT WRONG?</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>No pre-start port validation on payment-processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ACTION ITEMS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Add port check to systemd ExecStartPre</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Next sprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CloudWatch ServiceDown alarm → on-call</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SRE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>This week</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LESSONS LEARNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Validate port availability before service restart</t>
         </is>
       </c>
     </row>
@@ -940,13 +1601,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>RB-AWS-001</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>RUNBOOK / SOP</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Document ID: RB-AWS-001</t>
         </is>
       </c>
     </row>
@@ -965,12 +1635,157 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>STEP 4</t>
+          <t>TRIGGER</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sudo ss -tulpn | grep 8080</t>
+          <t>CloudWatch Alarm: PaymentProcessor-ServiceDown; user reports transactions failing</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>STEP 1 — ACKNOWLEDGE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Note time; check Lab3-SLA-Dashboard for impact duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>STEP 2 — CHECK SERVICE STATUS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>systemctl status payment-processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>STEP 3 — CHECK LOGS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>sudo journalctl -u payment-processor -n 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>STEP 4 — CHECK PORT CONFLICT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sudo ss -tulpn | grep 8080; pgrep -af rogue-process.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>STEP 5 — KILL CONFLICTING PROCESS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sudo kill -9 &lt;PID&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>STEP 6 — RESTART SERVICE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sudo systemctl reset-failed payment-processor; sudo systemctl restart payment-processor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>STEP 7 — VERIFY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>systemctl is-active payment-processor; curl -s -o /dev/null -w '%{http_code}' http://localhost:8080</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>STEP 8 — CLOSE INCIDENT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Document root cause; update resolution time; close ticket</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ESCALATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L2 Support</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>_______________</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L3 Support</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>_______________</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>On-call Manager</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>_______________</t>
         </is>
       </c>
     </row>

</xml_diff>